<commit_message>
Fix image loading and Vercel deployment
</commit_message>
<xml_diff>
--- a/data/timemap_data.xlsx
+++ b/data/timemap_data.xlsx
@@ -1033,7 +1033,7 @@
     <numFmt numFmtId="168" formatCode="d-mmmm-yy"/>
     <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1120,11 +1120,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <u/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -1143,7 +1138,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1214,11 +1209,10 @@
     <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -5770,7 +5764,7 @@
         <v>Honduran Government Enacts New General Mining Law</v>
       </c>
       <c r="C2" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C2), "", CONCAT("http://localhost:4040/images/", Sources!C2))</f>
+        <f>IF(ISBLANK(Sources!C2), "", CONCAT("images/", Sources!C2))</f>
         <v/>
       </c>
       <c r="D2" s="20" t="str">
@@ -5778,15 +5772,15 @@
         <v>Honduran Government Enacts New General Mining Law</v>
       </c>
       <c r="E2" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E2), "", CONCAT("http://localhost:4040/", Sources!E2))</f>
+        <f>IF(ISBLANK(Sources!E2), "", CONCAT("", Sources!E2))</f>
         <v/>
       </c>
       <c r="F2" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F2), "", CONCAT("http://localhost:4040/", Sources!F2))</f>
+        <f>IF(ISBLANK(Sources!F2), "", CONCAT("", Sources!F2))</f>
         <v/>
       </c>
       <c r="G2" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G2), "", CONCAT("http://localhost:4040/", Sources!G2))</f>
+        <f>IF(ISBLANK(Sources!G2), "", CONCAT("", Sources!G2))</f>
         <v/>
       </c>
       <c r="H2" s="20"/>
@@ -5801,7 +5795,7 @@
         <v>Honduras Reduces Carlos Escaleras Mejía National Park Protected Area</v>
       </c>
       <c r="C3" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C3), "", CONCAT("http://localhost:4040/images/", Sources!C3))</f>
+        <f>IF(ISBLANK(Sources!C3), "", CONCAT("images/", Sources!C3))</f>
         <v/>
       </c>
       <c r="D3" s="20" t="str">
@@ -5809,15 +5803,15 @@
         <v>Honduras Reduces Carlos Escaleras Mejía National Park Protected Area</v>
       </c>
       <c r="E3" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E3), "", CONCAT("http://localhost:4040/", Sources!E3))</f>
-        <v>http://localhost:4040/images/231213.png</v>
+        <f>IF(ISBLANK(Sources!E3), "", CONCAT("", Sources!E3))</f>
+        <v>images/231213.png</v>
       </c>
       <c r="F3" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F3), "", CONCAT("http://localhost:4040/", Sources!F3))</f>
+        <f>IF(ISBLANK(Sources!F3), "", CONCAT("", Sources!F3))</f>
         <v/>
       </c>
       <c r="G3" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G3), "", CONCAT("http://localhost:4040/", Sources!G3))</f>
+        <f>IF(ISBLANK(Sources!G3), "", CONCAT("", Sources!G3))</f>
         <v/>
       </c>
       <c r="H3" s="20"/>
@@ -5832,7 +5826,7 @@
         <v>Los Pinares Granted Mining License in National Park</v>
       </c>
       <c r="C4" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C4), "", CONCAT("http://localhost:4040/images/", Sources!C4))</f>
+        <f>IF(ISBLANK(Sources!C4), "", CONCAT("images/", Sources!C4))</f>
         <v/>
       </c>
       <c r="D4" s="20" t="str">
@@ -5840,15 +5834,15 @@
         <v>Los Pinares Granted Mining License in National Park</v>
       </c>
       <c r="E4" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E4), "", CONCAT("http://localhost:4040/", Sources!E4))</f>
-        <v>http://localhost:4040/images/28012014.png</v>
+        <f>IF(ISBLANK(Sources!E4), "", CONCAT("", Sources!E4))</f>
+        <v>images/28012014.png</v>
       </c>
       <c r="F4" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F4), "", CONCAT("http://localhost:4040/", Sources!F4))</f>
+        <f>IF(ISBLANK(Sources!F4), "", CONCAT("", Sources!F4))</f>
         <v/>
       </c>
       <c r="G4" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G4), "", CONCAT("http://localhost:4040/", Sources!G4))</f>
+        <f>IF(ISBLANK(Sources!G4), "", CONCAT("", Sources!G4))</f>
         <v/>
       </c>
       <c r="H4" s="20"/>
@@ -5863,7 +5857,7 @@
         <v>ECOTEK Obtains License for Iron Pelletizing Plant</v>
       </c>
       <c r="C5" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C5), "", CONCAT("http://localhost:4040/images/", Sources!C5))</f>
+        <f>IF(ISBLANK(Sources!C5), "", CONCAT("images/", Sources!C5))</f>
         <v/>
       </c>
       <c r="D5" s="20" t="str">
@@ -5871,15 +5865,15 @@
         <v>ECOTEK Obtains License for Iron Pelletizing Plant</v>
       </c>
       <c r="E5" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E5), "", CONCAT("http://localhost:4040/", Sources!E5))</f>
+        <f>IF(ISBLANK(Sources!E5), "", CONCAT("", Sources!E5))</f>
         <v/>
       </c>
       <c r="F5" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F5), "", CONCAT("http://localhost:4040/", Sources!F5))</f>
+        <f>IF(ISBLANK(Sources!F5), "", CONCAT("", Sources!F5))</f>
         <v/>
       </c>
       <c r="G5" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G5), "", CONCAT("http://localhost:4040/", Sources!G5))</f>
+        <f>IF(ISBLANK(Sources!G5), "", CONCAT("", Sources!G5))</f>
         <v/>
       </c>
       <c r="H5" s="20"/>
@@ -5894,7 +5888,7 @@
         <v>Guapinol River Contamination Documented by Residents</v>
       </c>
       <c r="C6" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C6), "", CONCAT("http://localhost:4040/images/", Sources!C6))</f>
+        <f>IF(ISBLANK(Sources!C6), "", CONCAT("images/", Sources!C6))</f>
         <v/>
       </c>
       <c r="D6" s="20" t="str">
@@ -5902,16 +5896,16 @@
         <v>Guapinol River Contamination Documented by Residents</v>
       </c>
       <c r="E6" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E6), "", CONCAT("http://localhost:4040/", Sources!E6))</f>
-        <v>http://localhost:4040/images/26042018.jpg</v>
-      </c>
-      <c r="F6" s="32" t="str">
-        <f>IF(ISBLANK(Sources!F6), "", CONCAT("http://localhost:4040/", Sources!F6))</f>
-        <v>http://localhost:4040/images/26042018a.jpg</v>
-      </c>
-      <c r="G6" s="32" t="str">
-        <f>IF(ISBLANK(Sources!G6), "", CONCAT("http://localhost:4040/", Sources!G6))</f>
-        <v>http://localhost:4040/images/26042018b.jpg</v>
+        <f>IF(ISBLANK(Sources!E6), "", CONCAT("", Sources!E6))</f>
+        <v>images/26042018.jpg</v>
+      </c>
+      <c r="F6" s="20" t="str">
+        <f>IF(ISBLANK(Sources!F6), "", CONCAT("", Sources!F6))</f>
+        <v>images/26042018a.jpg</v>
+      </c>
+      <c r="G6" s="20" t="str">
+        <f>IF(ISBLANK(Sources!G6), "", CONCAT("", Sources!G6))</f>
+        <v>images/26042018b.jpg</v>
       </c>
       <c r="H6" s="20"/>
     </row>
@@ -5925,7 +5919,7 @@
         <v>Community Meeting Organized to Discuss Mining Project</v>
       </c>
       <c r="C7" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C7), "", CONCAT("http://localhost:4040/images/", Sources!C7))</f>
+        <f>IF(ISBLANK(Sources!C7), "", CONCAT("images/", Sources!C7))</f>
         <v/>
       </c>
       <c r="D7" s="20" t="str">
@@ -5933,15 +5927,15 @@
         <v>Community Meeting Organized to Discuss Mining Project</v>
       </c>
       <c r="E7" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E7), "", CONCAT("http://localhost:4040/", Sources!E7))</f>
-        <v>http://localhost:4040/images/07052018.jpg</v>
+        <f>IF(ISBLANK(Sources!E7), "", CONCAT("", Sources!E7))</f>
+        <v>images/07052018.jpg</v>
       </c>
       <c r="F7" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F7), "", CONCAT("http://localhost:4040/", Sources!F7))</f>
+        <f>IF(ISBLANK(Sources!F7), "", CONCAT("", Sources!F7))</f>
         <v/>
       </c>
       <c r="G7" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G7), "", CONCAT("http://localhost:4040/", Sources!G7))</f>
+        <f>IF(ISBLANK(Sources!G7), "", CONCAT("", Sources!G7))</f>
         <v/>
       </c>
       <c r="H7" s="20"/>
@@ -5956,7 +5950,7 @@
         <v>Peaceful Demonstration at Caja Rural Meeting</v>
       </c>
       <c r="C8" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C8), "", CONCAT("http://localhost:4040/images/", Sources!C8))</f>
+        <f>IF(ISBLANK(Sources!C8), "", CONCAT("images/", Sources!C8))</f>
         <v/>
       </c>
       <c r="D8" s="20" t="str">
@@ -5964,16 +5958,16 @@
         <v>Peaceful Demonstration at Caja Rural</v>
       </c>
       <c r="E8" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E8), "", CONCAT("http://localhost:4040/", Sources!E8))</f>
-        <v>http://localhost:4040/images/10052018.jpg</v>
-      </c>
-      <c r="F8" s="32" t="str">
-        <f>IF(ISBLANK(Sources!F8), "", CONCAT("http://localhost:4040/", Sources!F8))</f>
-        <v>http://localhost:4040/images/10052018a.jpg</v>
-      </c>
-      <c r="G8" s="32" t="str">
-        <f>IF(ISBLANK(Sources!G8), "", CONCAT("http://localhost:4040/", Sources!G8))</f>
-        <v>http://localhost:4040/images/10052018b.jpg</v>
+        <f>IF(ISBLANK(Sources!E8), "", CONCAT("", Sources!E8))</f>
+        <v>images/10052018.jpg</v>
+      </c>
+      <c r="F8" s="20" t="str">
+        <f>IF(ISBLANK(Sources!F8), "", CONCAT("", Sources!F8))</f>
+        <v>images/10052018a.jpg</v>
+      </c>
+      <c r="G8" s="20" t="str">
+        <f>IF(ISBLANK(Sources!G8), "", CONCAT("", Sources!G8))</f>
+        <v>images/10052018b.jpg</v>
       </c>
       <c r="H8" s="20"/>
     </row>
@@ -5987,7 +5981,7 @@
         <v>Further River Contamination Evidence Circulated</v>
       </c>
       <c r="C9" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C9), "", CONCAT("http://localhost:4040/images/", Sources!C9))</f>
+        <f>IF(ISBLANK(Sources!C9), "", CONCAT("images/", Sources!C9))</f>
         <v/>
       </c>
       <c r="D9" s="20" t="str">
@@ -5995,15 +5989,15 @@
         <v>Further River Contamination Evidence Circulated</v>
       </c>
       <c r="E9" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E9), "", CONCAT("http://localhost:4040/", Sources!E9))</f>
-        <v>http://localhost:4040/images/30072018.jpg</v>
-      </c>
-      <c r="F9" s="32" t="str">
-        <f>IF(ISBLANK(Sources!F9), "", CONCAT("http://localhost:4040/", Sources!F9))</f>
-        <v>http://localhost:4040/images/30072018a.mp4</v>
+        <f>IF(ISBLANK(Sources!E9), "", CONCAT("", Sources!E9))</f>
+        <v>images/30072018.jpg</v>
+      </c>
+      <c r="F9" s="20" t="str">
+        <f>IF(ISBLANK(Sources!F9), "", CONCAT("", Sources!F9))</f>
+        <v>images/30072018a.mp4</v>
       </c>
       <c r="G9" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G9), "", CONCAT("http://localhost:4040/", Sources!G9))</f>
+        <f>IF(ISBLANK(Sources!G9), "", CONCAT("", Sources!G9))</f>
         <v/>
       </c>
       <c r="H9" s="20"/>
@@ -6018,7 +6012,7 @@
         <v>Guapinol Encampment Established to Defend Water</v>
       </c>
       <c r="C10" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C10), "", CONCAT("http://localhost:4040/images/", Sources!C10))</f>
+        <f>IF(ISBLANK(Sources!C10), "", CONCAT("images/", Sources!C10))</f>
         <v/>
       </c>
       <c r="D10" s="20" t="str">
@@ -6026,16 +6020,16 @@
         <v>Guapinol Encampment Established to Defend Water</v>
       </c>
       <c r="E10" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E10), "", CONCAT("http://localhost:4040/", Sources!E10))</f>
-        <v>http://localhost:4040/images/01082018.jpg</v>
-      </c>
-      <c r="F10" s="32" t="str">
-        <f>IF(ISBLANK(Sources!F10), "", CONCAT("http://localhost:4040/", Sources!F10))</f>
-        <v>http://localhost:4040/images/01082018a.jpg</v>
-      </c>
-      <c r="G10" s="32" t="str">
-        <f>IF(ISBLANK(Sources!G10), "", CONCAT("http://localhost:4040/", Sources!G10))</f>
-        <v>http://localhost:4040/images/01082018b.jpg</v>
+        <f>IF(ISBLANK(Sources!E10), "", CONCAT("", Sources!E10))</f>
+        <v>images/01082018.jpg</v>
+      </c>
+      <c r="F10" s="20" t="str">
+        <f>IF(ISBLANK(Sources!F10), "", CONCAT("", Sources!F10))</f>
+        <v>images/01082018a.jpg</v>
+      </c>
+      <c r="G10" s="20" t="str">
+        <f>IF(ISBLANK(Sources!G10), "", CONCAT("", Sources!G10))</f>
+        <v>images/01082018b.jpg</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -6048,7 +6042,7 @@
         <v>Security Official Shoots Protester During Dispute</v>
       </c>
       <c r="C11" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C11), "", CONCAT("http://localhost:4040/images/", Sources!C11))</f>
+        <f>IF(ISBLANK(Sources!C11), "", CONCAT("images/", Sources!C11))</f>
         <v/>
       </c>
       <c r="D11" s="20" t="str">
@@ -6056,15 +6050,15 @@
         <v>Security Official Shoots Protester During Dispute</v>
       </c>
       <c r="E11" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E11), "", CONCAT("http://localhost:4040/", Sources!E11))</f>
-        <v>http://localhost:4040/images/07092018.jpg</v>
+        <f>IF(ISBLANK(Sources!E11), "", CONCAT("", Sources!E11))</f>
+        <v>images/07092018.jpg</v>
       </c>
       <c r="F11" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F11), "", CONCAT("http://localhost:4040/", Sources!F11))</f>
+        <f>IF(ISBLANK(Sources!F11), "", CONCAT("", Sources!F11))</f>
         <v/>
       </c>
       <c r="G11" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G11), "", CONCAT("http://localhost:4040/", Sources!G11))</f>
+        <f>IF(ISBLANK(Sources!G11), "", CONCAT("", Sources!G11))</f>
         <v/>
       </c>
     </row>
@@ -6078,7 +6072,7 @@
         <v>Arrest Warrants Issued for Eighteen Community Members</v>
       </c>
       <c r="C12" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C12), "", CONCAT("http://localhost:4040/images/", Sources!C12))</f>
+        <f>IF(ISBLANK(Sources!C12), "", CONCAT("images/", Sources!C12))</f>
         <v/>
       </c>
       <c r="D12" s="20" t="str">
@@ -6086,15 +6080,15 @@
         <v>Arrest Warrants Issued for Eighteen Community Members</v>
       </c>
       <c r="E12" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E12), "", CONCAT("http://localhost:4040/", Sources!E12))</f>
+        <f>IF(ISBLANK(Sources!E12), "", CONCAT("", Sources!E12))</f>
         <v/>
       </c>
       <c r="F12" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F12), "", CONCAT("http://localhost:4040/", Sources!F12))</f>
+        <f>IF(ISBLANK(Sources!F12), "", CONCAT("", Sources!F12))</f>
         <v/>
       </c>
       <c r="G12" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G12), "", CONCAT("http://localhost:4040/", Sources!G12))</f>
+        <f>IF(ISBLANK(Sources!G12), "", CONCAT("", Sources!G12))</f>
         <v/>
       </c>
     </row>
@@ -6108,7 +6102,7 @@
         <v>Police and Military Evict Encampment with Violence</v>
       </c>
       <c r="C13" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C13), "", CONCAT("http://localhost:4040/images/", Sources!C13))</f>
+        <f>IF(ISBLANK(Sources!C13), "", CONCAT("images/", Sources!C13))</f>
         <v/>
       </c>
       <c r="D13" s="20" t="str">
@@ -6116,15 +6110,15 @@
         <v>Police and Military Evict Encampment with Violence</v>
       </c>
       <c r="E13" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E13), "", CONCAT("http://localhost:4040/", Sources!E13))</f>
-        <v>http://localhost:4040/images/27102018.mp4</v>
+        <f>IF(ISBLANK(Sources!E13), "", CONCAT("", Sources!E13))</f>
+        <v>images/27102018.mp4</v>
       </c>
       <c r="F13" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F13), "", CONCAT("http://localhost:4040/", Sources!F13))</f>
+        <f>IF(ISBLANK(Sources!F13), "", CONCAT("", Sources!F13))</f>
         <v/>
       </c>
       <c r="G13" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G13), "", CONCAT("http://localhost:4040/", Sources!G13))</f>
+        <f>IF(ISBLANK(Sources!G13), "", CONCAT("", Sources!G13))</f>
         <v/>
       </c>
     </row>
@@ -6138,7 +6132,7 @@
         <v>Thirteen Community Members Appear Before Court</v>
       </c>
       <c r="C14" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C14), "", CONCAT("http://localhost:4040/images/", Sources!C14))</f>
+        <f>IF(ISBLANK(Sources!C14), "", CONCAT("images/", Sources!C14))</f>
         <v/>
       </c>
       <c r="D14" s="20" t="str">
@@ -6146,15 +6140,15 @@
         <v>Thirteen Community Members Appear Before Court</v>
       </c>
       <c r="E14" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E14), "", CONCAT("http://localhost:4040/", Sources!E14))</f>
+        <f>IF(ISBLANK(Sources!E14), "", CONCAT("", Sources!E14))</f>
         <v/>
       </c>
       <c r="F14" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F14), "", CONCAT("http://localhost:4040/", Sources!F14))</f>
+        <f>IF(ISBLANK(Sources!F14), "", CONCAT("", Sources!F14))</f>
         <v/>
       </c>
       <c r="G14" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G14), "", CONCAT("http://localhost:4040/", Sources!G14))</f>
+        <f>IF(ISBLANK(Sources!G14), "", CONCAT("", Sources!G14))</f>
         <v/>
       </c>
     </row>
@@ -6168,7 +6162,7 @@
         <v>Constitutional Challenge Filed Against Decree 252-2013</v>
       </c>
       <c r="C15" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C15), "", CONCAT("http://localhost:4040/images/", Sources!C15))</f>
+        <f>IF(ISBLANK(Sources!C15), "", CONCAT("images/", Sources!C15))</f>
         <v/>
       </c>
       <c r="D15" s="20" t="str">
@@ -6176,15 +6170,15 @@
         <v>Constitutional Challenge Filed Against Decree 252-2013</v>
       </c>
       <c r="E15" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E15), "", CONCAT("http://localhost:4040/", Sources!E15))</f>
+        <f>IF(ISBLANK(Sources!E15), "", CONCAT("", Sources!E15))</f>
         <v/>
       </c>
       <c r="F15" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F15), "", CONCAT("http://localhost:4040/", Sources!F15))</f>
+        <f>IF(ISBLANK(Sources!F15), "", CONCAT("", Sources!F15))</f>
         <v/>
       </c>
       <c r="G15" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G15), "", CONCAT("http://localhost:4040/", Sources!G15))</f>
+        <f>IF(ISBLANK(Sources!G15), "", CONCAT("", Sources!G15))</f>
         <v/>
       </c>
     </row>
@@ -6198,7 +6192,7 @@
         <v>Charges Dismissed Against Thirteen Defenders</v>
       </c>
       <c r="C16" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C16), "", CONCAT("http://localhost:4040/images/", Sources!C16))</f>
+        <f>IF(ISBLANK(Sources!C16), "", CONCAT("images/", Sources!C16))</f>
         <v/>
       </c>
       <c r="D16" s="20" t="str">
@@ -6206,15 +6200,15 @@
         <v>Charges Dismissed Against Thirteen Defenders</v>
       </c>
       <c r="E16" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E16), "", CONCAT("http://localhost:4040/", Sources!E16))</f>
+        <f>IF(ISBLANK(Sources!E16), "", CONCAT("", Sources!E16))</f>
         <v/>
       </c>
       <c r="F16" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F16), "", CONCAT("http://localhost:4040/", Sources!F16))</f>
+        <f>IF(ISBLANK(Sources!F16), "", CONCAT("", Sources!F16))</f>
         <v/>
       </c>
       <c r="G16" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G16), "", CONCAT("http://localhost:4040/", Sources!G16))</f>
+        <f>IF(ISBLANK(Sources!G16), "", CONCAT("", Sources!G16))</f>
         <v/>
       </c>
     </row>
@@ -6228,7 +6222,7 @@
         <v>Detained Protesters Released</v>
       </c>
       <c r="C17" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C17), "", CONCAT("http://localhost:4040/images/", Sources!C17))</f>
+        <f>IF(ISBLANK(Sources!C17), "", CONCAT("images/", Sources!C17))</f>
         <v/>
       </c>
       <c r="D17" s="20" t="str">
@@ -6236,15 +6230,15 @@
         <v>Detained Protesters Released</v>
       </c>
       <c r="E17" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E17), "", CONCAT("http://localhost:4040/", Sources!E17))</f>
-        <v>http://localhost:4040/images/06032019.jpg</v>
+        <f>IF(ISBLANK(Sources!E17), "", CONCAT("", Sources!E17))</f>
+        <v>images/06032019.jpg</v>
       </c>
       <c r="F17" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F17), "", CONCAT("http://localhost:4040/", Sources!F17))</f>
+        <f>IF(ISBLANK(Sources!F17), "", CONCAT("", Sources!F17))</f>
         <v/>
       </c>
       <c r="G17" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G17), "", CONCAT("http://localhost:4040/", Sources!G17))</f>
+        <f>IF(ISBLANK(Sources!G17), "", CONCAT("", Sources!G17))</f>
         <v/>
       </c>
     </row>
@@ -6258,7 +6252,7 @@
         <v>Seven Additional Community Members Appear in Court</v>
       </c>
       <c r="C18" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C18), "", CONCAT("http://localhost:4040/images/", Sources!C18))</f>
+        <f>IF(ISBLANK(Sources!C18), "", CONCAT("images/", Sources!C18))</f>
         <v/>
       </c>
       <c r="D18" s="20" t="str">
@@ -6266,15 +6260,15 @@
         <v>Seven Additional Community Members Appear in Court</v>
       </c>
       <c r="E18" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E18), "", CONCAT("http://localhost:4040/", Sources!E18))</f>
-        <v>http://localhost:4040/images/26082019.mp4</v>
+        <f>IF(ISBLANK(Sources!E18), "", CONCAT("", Sources!E18))</f>
+        <v>images/26082019.mp4</v>
       </c>
       <c r="F18" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F18), "", CONCAT("http://localhost:4040/", Sources!F18))</f>
+        <f>IF(ISBLANK(Sources!F18), "", CONCAT("", Sources!F18))</f>
         <v/>
       </c>
       <c r="G18" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G18), "", CONCAT("http://localhost:4040/", Sources!G18))</f>
+        <f>IF(ISBLANK(Sources!G18), "", CONCAT("", Sources!G18))</f>
         <v/>
       </c>
     </row>
@@ -6288,7 +6282,7 @@
         <v>Environmental Defender Roberto Argueta Assassinated</v>
       </c>
       <c r="C19" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C19), "", CONCAT("http://localhost:4040/images/", Sources!C19))</f>
+        <f>IF(ISBLANK(Sources!C19), "", CONCAT("images/", Sources!C19))</f>
         <v/>
       </c>
       <c r="D19" s="20" t="str">
@@ -6296,15 +6290,15 @@
         <v>Environmental Defender Roberto Argueta Assassinated</v>
       </c>
       <c r="E19" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E19), "", CONCAT("http://localhost:4040/", Sources!E19))</f>
-        <v>http://localhost:4040/images/28082019.jpg</v>
+        <f>IF(ISBLANK(Sources!E19), "", CONCAT("", Sources!E19))</f>
+        <v>images/28082019.jpg</v>
       </c>
       <c r="F19" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F19), "", CONCAT("http://localhost:4040/", Sources!F19))</f>
+        <f>IF(ISBLANK(Sources!F19), "", CONCAT("", Sources!F19))</f>
         <v/>
       </c>
       <c r="G19" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G19), "", CONCAT("http://localhost:4040/", Sources!G19))</f>
+        <f>IF(ISBLANK(Sources!G19), "", CONCAT("", Sources!G19))</f>
         <v/>
       </c>
     </row>
@@ -6318,7 +6312,7 @@
         <v>Temporary Dismissal Granted to Arnold Alemán</v>
       </c>
       <c r="C20" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C20), "", CONCAT("http://localhost:4040/images/", Sources!C20))</f>
+        <f>IF(ISBLANK(Sources!C20), "", CONCAT("images/", Sources!C20))</f>
         <v/>
       </c>
       <c r="D20" s="20" t="str">
@@ -6326,15 +6320,15 @@
         <v>Temporary Dismissal Granted to Arnold Alemán</v>
       </c>
       <c r="E20" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E20), "", CONCAT("http://localhost:4040/", Sources!E20))</f>
+        <f>IF(ISBLANK(Sources!E20), "", CONCAT("", Sources!E20))</f>
         <v/>
       </c>
       <c r="F20" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F20), "", CONCAT("http://localhost:4040/", Sources!F20))</f>
+        <f>IF(ISBLANK(Sources!F20), "", CONCAT("", Sources!F20))</f>
         <v/>
       </c>
       <c r="G20" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G20), "", CONCAT("http://localhost:4040/", Sources!G20))</f>
+        <f>IF(ISBLANK(Sources!G20), "", CONCAT("", Sources!G20))</f>
         <v/>
       </c>
     </row>
@@ -6348,7 +6342,7 @@
         <v>Nine Environmental Defenders Placed in Pretrial Detention</v>
       </c>
       <c r="C21" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C21), "", CONCAT("http://localhost:4040/images/", Sources!C21))</f>
+        <f>IF(ISBLANK(Sources!C21), "", CONCAT("images/", Sources!C21))</f>
         <v/>
       </c>
       <c r="D21" s="20" t="str">
@@ -6356,15 +6350,15 @@
         <v>Nine Environmental Defenders Placed in Pretrial Detention</v>
       </c>
       <c r="E21" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E21), "", CONCAT("http://localhost:4040/", Sources!E21))</f>
-        <v>http://localhost:4040/images/01092019.mp4</v>
+        <f>IF(ISBLANK(Sources!E21), "", CONCAT("", Sources!E21))</f>
+        <v>images/01092019.mp4</v>
       </c>
       <c r="F21" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F21), "", CONCAT("http://localhost:4040/", Sources!F21))</f>
+        <f>IF(ISBLANK(Sources!F21), "", CONCAT("", Sources!F21))</f>
         <v/>
       </c>
       <c r="G21" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G21), "", CONCAT("http://localhost:4040/", Sources!G21))</f>
+        <f>IF(ISBLANK(Sources!G21), "", CONCAT("", Sources!G21))</f>
         <v/>
       </c>
     </row>
@@ -6378,7 +6372,7 @@
         <v>Court Rejects Habeas Corpus Petition</v>
       </c>
       <c r="C22" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C22), "", CONCAT("http://localhost:4040/images/", Sources!C22))</f>
+        <f>IF(ISBLANK(Sources!C22), "", CONCAT("images/", Sources!C22))</f>
         <v/>
       </c>
       <c r="D22" s="20" t="str">
@@ -6386,15 +6380,15 @@
         <v>Court Rejects Habeas Corpus Petition</v>
       </c>
       <c r="E22" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E22), "", CONCAT("http://localhost:4040/", Sources!E22))</f>
+        <f>IF(ISBLANK(Sources!E22), "", CONCAT("", Sources!E22))</f>
         <v/>
       </c>
       <c r="F22" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F22), "", CONCAT("http://localhost:4040/", Sources!F22))</f>
+        <f>IF(ISBLANK(Sources!F22), "", CONCAT("", Sources!F22))</f>
         <v/>
       </c>
       <c r="G22" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G22), "", CONCAT("http://localhost:4040/", Sources!G22))</f>
+        <f>IF(ISBLANK(Sources!G22), "", CONCAT("", Sources!G22))</f>
         <v/>
       </c>
     </row>
@@ -6408,7 +6402,7 @@
         <v>Pretrial Detention Extended for Guapinol Activists</v>
       </c>
       <c r="C23" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C23), "", CONCAT("http://localhost:4040/images/", Sources!C23))</f>
+        <f>IF(ISBLANK(Sources!C23), "", CONCAT("images/", Sources!C23))</f>
         <v/>
       </c>
       <c r="D23" s="20" t="str">
@@ -6416,15 +6410,15 @@
         <v>Pretrial Detention Extended for Guapinol Activists</v>
       </c>
       <c r="E23" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E23), "", CONCAT("http://localhost:4040/", Sources!E23))</f>
+        <f>IF(ISBLANK(Sources!E23), "", CONCAT("", Sources!E23))</f>
         <v/>
       </c>
       <c r="F23" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F23), "", CONCAT("http://localhost:4040/", Sources!F23))</f>
+        <f>IF(ISBLANK(Sources!F23), "", CONCAT("", Sources!F23))</f>
         <v/>
       </c>
       <c r="G23" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G23), "", CONCAT("http://localhost:4040/", Sources!G23))</f>
+        <f>IF(ISBLANK(Sources!G23), "", CONCAT("", Sources!G23))</f>
         <v/>
       </c>
     </row>
@@ -6438,7 +6432,7 @@
         <v>Break-ins Reported at COPA Office</v>
       </c>
       <c r="C24" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C24), "", CONCAT("http://localhost:4040/images/", Sources!C24))</f>
+        <f>IF(ISBLANK(Sources!C24), "", CONCAT("images/", Sources!C24))</f>
         <v/>
       </c>
       <c r="D24" s="20" t="str">
@@ -6446,15 +6440,15 @@
         <v>Break-ins Reported at COPA Office</v>
       </c>
       <c r="E24" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E24), "", CONCAT("http://localhost:4040/", Sources!E24))</f>
+        <f>IF(ISBLANK(Sources!E24), "", CONCAT("", Sources!E24))</f>
         <v/>
       </c>
       <c r="F24" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F24), "", CONCAT("http://localhost:4040/", Sources!F24))</f>
+        <f>IF(ISBLANK(Sources!F24), "", CONCAT("", Sources!F24))</f>
         <v/>
       </c>
       <c r="G24" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G24), "", CONCAT("http://localhost:4040/", Sources!G24))</f>
+        <f>IF(ISBLANK(Sources!G24), "", CONCAT("", Sources!G24))</f>
         <v/>
       </c>
     </row>
@@ -6468,7 +6462,7 @@
         <v>CEJIL Submits Amicus Brief to Court of Appeals</v>
       </c>
       <c r="C25" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C25), "", CONCAT("http://localhost:4040/images/", Sources!C25))</f>
+        <f>IF(ISBLANK(Sources!C25), "", CONCAT("images/", Sources!C25))</f>
         <v/>
       </c>
       <c r="D25" s="20" t="str">
@@ -6476,15 +6470,15 @@
         <v>CEJIL Submits Amicus Brief to Court of Appeals</v>
       </c>
       <c r="E25" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E25), "", CONCAT("http://localhost:4040/", Sources!E25))</f>
+        <f>IF(ISBLANK(Sources!E25), "", CONCAT("", Sources!E25))</f>
         <v/>
       </c>
       <c r="F25" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F25), "", CONCAT("http://localhost:4040/", Sources!F25))</f>
+        <f>IF(ISBLANK(Sources!F25), "", CONCAT("", Sources!F25))</f>
         <v/>
       </c>
       <c r="G25" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G25), "", CONCAT("http://localhost:4040/", Sources!G25))</f>
+        <f>IF(ISBLANK(Sources!G25), "", CONCAT("", Sources!G25))</f>
         <v/>
       </c>
     </row>
@@ -6498,7 +6492,7 @@
         <v>Second Habeas Corpus Petition Filed with Supreme Court</v>
       </c>
       <c r="C26" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C26), "", CONCAT("http://localhost:4040/images/", Sources!C26))</f>
+        <f>IF(ISBLANK(Sources!C26), "", CONCAT("images/", Sources!C26))</f>
         <v/>
       </c>
       <c r="D26" s="20" t="str">
@@ -6506,15 +6500,15 @@
         <v>Second Habeas Corpus Petition Filed with Supreme Court</v>
       </c>
       <c r="E26" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E26), "", CONCAT("http://localhost:4040/", Sources!E26))</f>
+        <f>IF(ISBLANK(Sources!E26), "", CONCAT("", Sources!E26))</f>
         <v/>
       </c>
       <c r="F26" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F26), "", CONCAT("http://localhost:4040/", Sources!F26))</f>
+        <f>IF(ISBLANK(Sources!F26), "", CONCAT("", Sources!F26))</f>
         <v/>
       </c>
       <c r="G26" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G26), "", CONCAT("http://localhost:4040/", Sources!G26))</f>
+        <f>IF(ISBLANK(Sources!G26), "", CONCAT("", Sources!G26))</f>
         <v/>
       </c>
     </row>
@@ -6528,7 +6522,7 @@
         <v>Court of Appeals Overturns Previous Dismissal</v>
       </c>
       <c r="C27" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C27), "", CONCAT("http://localhost:4040/images/", Sources!C27))</f>
+        <f>IF(ISBLANK(Sources!C27), "", CONCAT("images/", Sources!C27))</f>
         <v/>
       </c>
       <c r="D27" s="20" t="str">
@@ -6536,15 +6530,15 @@
         <v>Court of Appeals Overturns Previous Dismissal</v>
       </c>
       <c r="E27" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E27), "", CONCAT("http://localhost:4040/", Sources!E27))</f>
+        <f>IF(ISBLANK(Sources!E27), "", CONCAT("", Sources!E27))</f>
         <v/>
       </c>
       <c r="F27" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F27), "", CONCAT("http://localhost:4040/", Sources!F27))</f>
+        <f>IF(ISBLANK(Sources!F27), "", CONCAT("", Sources!F27))</f>
         <v/>
       </c>
       <c r="G27" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G27), "", CONCAT("http://localhost:4040/", Sources!G27))</f>
+        <f>IF(ISBLANK(Sources!G27), "", CONCAT("", Sources!G27))</f>
         <v/>
       </c>
     </row>
@@ -6558,7 +6552,7 @@
         <v>Human Rights Ombudsperson Defends CMDBCP Members</v>
       </c>
       <c r="C28" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C28), "", CONCAT("http://localhost:4040/images/", Sources!C28))</f>
+        <f>IF(ISBLANK(Sources!C28), "", CONCAT("images/", Sources!C28))</f>
         <v/>
       </c>
       <c r="D28" s="20" t="str">
@@ -6566,15 +6560,15 @@
         <v>Human Rights Ombudsperson Defends CMDBCP Members</v>
       </c>
       <c r="E28" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E28), "", CONCAT("http://localhost:4040/", Sources!E28))</f>
+        <f>IF(ISBLANK(Sources!E28), "", CONCAT("", Sources!E28))</f>
         <v/>
       </c>
       <c r="F28" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F28), "", CONCAT("http://localhost:4040/", Sources!F28))</f>
+        <f>IF(ISBLANK(Sources!F28), "", CONCAT("", Sources!F28))</f>
         <v/>
       </c>
       <c r="G28" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G28), "", CONCAT("http://localhost:4040/", Sources!G28))</f>
+        <f>IF(ISBLANK(Sources!G28), "", CONCAT("", Sources!G28))</f>
         <v/>
       </c>
     </row>
@@ -6588,7 +6582,7 @@
         <v>Joaquin Morazan Erazo Assassinated</v>
       </c>
       <c r="C29" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C29), "", CONCAT("http://localhost:4040/images/", Sources!C29))</f>
+        <f>IF(ISBLANK(Sources!C29), "", CONCAT("images/", Sources!C29))</f>
         <v/>
       </c>
       <c r="D29" s="20" t="str">
@@ -6596,15 +6590,15 @@
         <v>Joaquin Morazan Erazo Assassinated</v>
       </c>
       <c r="E29" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E29), "", CONCAT("http://localhost:4040/", Sources!E29))</f>
-        <v>http://localhost:4040/images/13102020.jpg</v>
+        <f>IF(ISBLANK(Sources!E29), "", CONCAT("", Sources!E29))</f>
+        <v>images/13102020.jpg</v>
       </c>
       <c r="F29" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F29), "", CONCAT("http://localhost:4040/", Sources!F29))</f>
+        <f>IF(ISBLANK(Sources!F29), "", CONCAT("", Sources!F29))</f>
         <v/>
       </c>
       <c r="G29" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G29), "", CONCAT("http://localhost:4040/", Sources!G29))</f>
+        <f>IF(ISBLANK(Sources!G29), "", CONCAT("", Sources!G29))</f>
         <v/>
       </c>
     </row>
@@ -6618,7 +6612,7 @@
         <v>UN OHCHR Issues Report on Judicial System Misuse</v>
       </c>
       <c r="C30" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C30), "", CONCAT("http://localhost:4040/images/", Sources!C30))</f>
+        <f>IF(ISBLANK(Sources!C30), "", CONCAT("images/", Sources!C30))</f>
         <v/>
       </c>
       <c r="D30" s="20" t="str">
@@ -6626,15 +6620,15 @@
         <v>UN OHCHR Issues Report on Judicial System Misuse</v>
       </c>
       <c r="E30" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E30), "", CONCAT("http://localhost:4040/", Sources!E30))</f>
+        <f>IF(ISBLANK(Sources!E30), "", CONCAT("", Sources!E30))</f>
         <v/>
       </c>
       <c r="F30" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F30), "", CONCAT("http://localhost:4040/", Sources!F30))</f>
+        <f>IF(ISBLANK(Sources!F30), "", CONCAT("", Sources!F30))</f>
         <v/>
       </c>
       <c r="G30" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G30), "", CONCAT("http://localhost:4040/", Sources!G30))</f>
+        <f>IF(ISBLANK(Sources!G30), "", CONCAT("", Sources!G30))</f>
         <v/>
       </c>
     </row>
@@ -6648,7 +6642,7 @@
         <v>UN Working Group Declares Guapinol Eight Arbitrarily Detained</v>
       </c>
       <c r="C31" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C31), "", CONCAT("http://localhost:4040/images/", Sources!C31))</f>
+        <f>IF(ISBLANK(Sources!C31), "", CONCAT("images/", Sources!C31))</f>
         <v/>
       </c>
       <c r="D31" s="20" t="str">
@@ -6656,15 +6650,15 @@
         <v>UN Working Group Declares Guapinol Eight Arbitrarily Detained</v>
       </c>
       <c r="E31" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E31), "", CONCAT("http://localhost:4040/", Sources!E31))</f>
+        <f>IF(ISBLANK(Sources!E31), "", CONCAT("", Sources!E31))</f>
         <v/>
       </c>
       <c r="F31" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F31), "", CONCAT("http://localhost:4040/", Sources!F31))</f>
+        <f>IF(ISBLANK(Sources!F31), "", CONCAT("", Sources!F31))</f>
         <v/>
       </c>
       <c r="G31" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G31), "", CONCAT("http://localhost:4040/", Sources!G31))</f>
+        <f>IF(ISBLANK(Sources!G31), "", CONCAT("", Sources!G31))</f>
         <v/>
       </c>
     </row>
@@ -6678,7 +6672,7 @@
         <v>Preventive Detention Extended for Guapinol Eight</v>
       </c>
       <c r="C32" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C32), "", CONCAT("http://localhost:4040/images/", Sources!C32))</f>
+        <f>IF(ISBLANK(Sources!C32), "", CONCAT("images/", Sources!C32))</f>
         <v/>
       </c>
       <c r="D32" s="20" t="str">
@@ -6686,15 +6680,15 @@
         <v>Preventive Detention Extended for Guapinol Eight</v>
       </c>
       <c r="E32" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E32), "", CONCAT("http://localhost:4040/", Sources!E32))</f>
+        <f>IF(ISBLANK(Sources!E32), "", CONCAT("", Sources!E32))</f>
         <v/>
       </c>
       <c r="F32" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F32), "", CONCAT("http://localhost:4040/", Sources!F32))</f>
+        <f>IF(ISBLANK(Sources!F32), "", CONCAT("", Sources!F32))</f>
         <v/>
       </c>
       <c r="G32" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G32), "", CONCAT("http://localhost:4040/", Sources!G32))</f>
+        <f>IF(ISBLANK(Sources!G32), "", CONCAT("", Sources!G32))</f>
         <v/>
       </c>
     </row>
@@ -6708,7 +6702,7 @@
         <v>Trial Against Guapinol Eight Begins After Two Years</v>
       </c>
       <c r="C33" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C33), "", CONCAT("http://localhost:4040/images/", Sources!C33))</f>
+        <f>IF(ISBLANK(Sources!C33), "", CONCAT("images/", Sources!C33))</f>
         <v/>
       </c>
       <c r="D33" s="20" t="str">
@@ -6716,15 +6710,15 @@
         <v>Trial Against Guapinol Eight Begins After Two Years</v>
       </c>
       <c r="E33" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E33), "", CONCAT("http://localhost:4040/", Sources!E33))</f>
-        <v>http://localhost:4040/images/01122021.mp4</v>
+        <f>IF(ISBLANK(Sources!E33), "", CONCAT("", Sources!E33))</f>
+        <v>images/01122021.mp4</v>
       </c>
       <c r="F33" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F33), "", CONCAT("http://localhost:4040/", Sources!F33))</f>
+        <f>IF(ISBLANK(Sources!F33), "", CONCAT("", Sources!F33))</f>
         <v/>
       </c>
       <c r="G33" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G33), "", CONCAT("http://localhost:4040/", Sources!G33))</f>
+        <f>IF(ISBLANK(Sources!G33), "", CONCAT("", Sources!G33))</f>
         <v/>
       </c>
     </row>
@@ -6738,7 +6732,7 @@
         <v>Amnesty International Expresses Concerns About Trial</v>
       </c>
       <c r="C34" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C34), "", CONCAT("http://localhost:4040/images/", Sources!C34))</f>
+        <f>IF(ISBLANK(Sources!C34), "", CONCAT("images/", Sources!C34))</f>
         <v/>
       </c>
       <c r="D34" s="20" t="str">
@@ -6746,15 +6740,15 @@
         <v>Amnesty International Expresses Concerns About Trial</v>
       </c>
       <c r="E34" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E34), "", CONCAT("http://localhost:4040/", Sources!E34))</f>
-        <v>http://localhost:4040/images/11122021.jpg</v>
+        <f>IF(ISBLANK(Sources!E34), "", CONCAT("", Sources!E34))</f>
+        <v>images/11122021.jpg</v>
       </c>
       <c r="F34" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F34), "", CONCAT("http://localhost:4040/", Sources!F34))</f>
+        <f>IF(ISBLANK(Sources!F34), "", CONCAT("", Sources!F34))</f>
         <v/>
       </c>
       <c r="G34" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G34), "", CONCAT("http://localhost:4040/", Sources!G34))</f>
+        <f>IF(ISBLANK(Sources!G34), "", CONCAT("", Sources!G34))</f>
         <v/>
       </c>
     </row>
@@ -6768,7 +6762,7 @@
         <v>Court Finds Six Defendants Guilty of Multiple Crimes</v>
       </c>
       <c r="C35" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C35), "", CONCAT("http://localhost:4040/images/", Sources!C35))</f>
+        <f>IF(ISBLANK(Sources!C35), "", CONCAT("images/", Sources!C35))</f>
         <v/>
       </c>
       <c r="D35" s="20" t="str">
@@ -6776,15 +6770,15 @@
         <v>Court Finds Six Defendants Guilty of Multiple Crimes</v>
       </c>
       <c r="E35" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E35), "", CONCAT("http://localhost:4040/", Sources!E35))</f>
+        <f>IF(ISBLANK(Sources!E35), "", CONCAT("", Sources!E35))</f>
         <v/>
       </c>
       <c r="F35" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F35), "", CONCAT("http://localhost:4040/", Sources!F35))</f>
+        <f>IF(ISBLANK(Sources!F35), "", CONCAT("", Sources!F35))</f>
         <v/>
       </c>
       <c r="G35" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G35), "", CONCAT("http://localhost:4040/", Sources!G35))</f>
+        <f>IF(ISBLANK(Sources!G35), "", CONCAT("", Sources!G35))</f>
         <v/>
       </c>
     </row>
@@ -6798,7 +6792,7 @@
         <v>Supreme Court Declares Mistrial and Grants Injunctions</v>
       </c>
       <c r="C36" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C36), "", CONCAT("http://localhost:4040/images/", Sources!C36))</f>
+        <f>IF(ISBLANK(Sources!C36), "", CONCAT("images/", Sources!C36))</f>
         <v/>
       </c>
       <c r="D36" s="20" t="str">
@@ -6806,15 +6800,15 @@
         <v>Supreme Court Declares Mistrial and Grants Injunctions</v>
       </c>
       <c r="E36" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E36), "", CONCAT("http://localhost:4040/", Sources!E36))</f>
+        <f>IF(ISBLANK(Sources!E36), "", CONCAT("", Sources!E36))</f>
         <v/>
       </c>
       <c r="F36" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F36), "", CONCAT("http://localhost:4040/", Sources!F36))</f>
+        <f>IF(ISBLANK(Sources!F36), "", CONCAT("", Sources!F36))</f>
         <v/>
       </c>
       <c r="G36" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G36), "", CONCAT("http://localhost:4040/", Sources!G36))</f>
+        <f>IF(ISBLANK(Sources!G36), "", CONCAT("", Sources!G36))</f>
         <v/>
       </c>
     </row>
@@ -6828,7 +6822,7 @@
         <v>Environmental Defenders Released on Bail After 914 Days</v>
       </c>
       <c r="C37" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C37), "", CONCAT("http://localhost:4040/images/", Sources!C37))</f>
+        <f>IF(ISBLANK(Sources!C37), "", CONCAT("images/", Sources!C37))</f>
         <v/>
       </c>
       <c r="D37" s="20" t="str">
@@ -6836,15 +6830,15 @@
         <v>Environmental Defenders Released on Bail After 914 Days</v>
       </c>
       <c r="E37" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E37), "", CONCAT("http://localhost:4040/", Sources!E37))</f>
-        <v>http://localhost:4040/images/25022022.jpg</v>
+        <f>IF(ISBLANK(Sources!E37), "", CONCAT("", Sources!E37))</f>
+        <v>images/25022022.jpg</v>
       </c>
       <c r="F37" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F37), "", CONCAT("http://localhost:4040/", Sources!F37))</f>
+        <f>IF(ISBLANK(Sources!F37), "", CONCAT("", Sources!F37))</f>
         <v/>
       </c>
       <c r="G37" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G37), "", CONCAT("http://localhost:4040/", Sources!G37))</f>
+        <f>IF(ISBLANK(Sources!G37), "", CONCAT("", Sources!G37))</f>
         <v/>
       </c>
     </row>
@@ -6858,7 +6852,7 @@
         <v>Two Anti-Mining Activists Murdered in Guapinol</v>
       </c>
       <c r="C38" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C38), "", CONCAT("http://localhost:4040/images/", Sources!C38))</f>
+        <f>IF(ISBLANK(Sources!C38), "", CONCAT("images/", Sources!C38))</f>
         <v/>
       </c>
       <c r="D38" s="20" t="str">
@@ -6866,15 +6860,15 @@
         <v>Two Anti-Mining Activists Murdered in Guapinol</v>
       </c>
       <c r="E38" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E38), "", CONCAT("http://localhost:4040/", Sources!E38))</f>
-        <v>http://localhost:4040/images/07012023.jpg</v>
+        <f>IF(ISBLANK(Sources!E38), "", CONCAT("", Sources!E38))</f>
+        <v>images/07012023.jpg</v>
       </c>
       <c r="F38" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F38), "", CONCAT("http://localhost:4040/", Sources!F38))</f>
+        <f>IF(ISBLANK(Sources!F38), "", CONCAT("", Sources!F38))</f>
         <v/>
       </c>
       <c r="G38" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G38), "", CONCAT("http://localhost:4040/", Sources!G38))</f>
+        <f>IF(ISBLANK(Sources!G38), "", CONCAT("", Sources!G38))</f>
         <v/>
       </c>
     </row>
@@ -6888,7 +6882,7 @@
         <v>Six Activists Face Possible Further Prosecution</v>
       </c>
       <c r="C39" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C39), "", CONCAT("http://localhost:4040/images/", Sources!C39))</f>
+        <f>IF(ISBLANK(Sources!C39), "", CONCAT("images/", Sources!C39))</f>
         <v/>
       </c>
       <c r="D39" s="20" t="str">
@@ -6896,15 +6890,15 @@
         <v>Six Activists Face Possible Further Prosecution</v>
       </c>
       <c r="E39" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E39), "", CONCAT("http://localhost:4040/", Sources!E39))</f>
+        <f>IF(ISBLANK(Sources!E39), "", CONCAT("", Sources!E39))</f>
         <v/>
       </c>
       <c r="F39" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F39), "", CONCAT("http://localhost:4040/", Sources!F39))</f>
+        <f>IF(ISBLANK(Sources!F39), "", CONCAT("", Sources!F39))</f>
         <v/>
       </c>
       <c r="G39" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G39), "", CONCAT("http://localhost:4040/", Sources!G39))</f>
+        <f>IF(ISBLANK(Sources!G39), "", CONCAT("", Sources!G39))</f>
         <v/>
       </c>
     </row>
@@ -6918,7 +6912,7 @@
         <v>Drones Reported Surveilling Activists' Homes</v>
       </c>
       <c r="C40" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C40), "", CONCAT("http://localhost:4040/images/", Sources!C40))</f>
+        <f>IF(ISBLANK(Sources!C40), "", CONCAT("images/", Sources!C40))</f>
         <v/>
       </c>
       <c r="D40" s="20" t="str">
@@ -6926,15 +6920,15 @@
         <v>Drones Reported Surveilling Activists' Homes</v>
       </c>
       <c r="E40" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E40), "", CONCAT("http://localhost:4040/", Sources!E40))</f>
-        <v>http://localhost:4040/images/21022023.jpg</v>
+        <f>IF(ISBLANK(Sources!E40), "", CONCAT("", Sources!E40))</f>
+        <v>images/21022023.jpg</v>
       </c>
       <c r="F40" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F40), "", CONCAT("http://localhost:4040/", Sources!F40))</f>
+        <f>IF(ISBLANK(Sources!F40), "", CONCAT("", Sources!F40))</f>
         <v/>
       </c>
       <c r="G40" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G40), "", CONCAT("http://localhost:4040/", Sources!G40))</f>
+        <f>IF(ISBLANK(Sources!G40), "", CONCAT("", Sources!G40))</f>
         <v/>
       </c>
     </row>
@@ -6948,7 +6942,7 @@
         <v>Oquelí Domínguez Murdered in Guapinol</v>
       </c>
       <c r="C41" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C41), "", CONCAT("http://localhost:4040/images/", Sources!C41))</f>
+        <f>IF(ISBLANK(Sources!C41), "", CONCAT("images/", Sources!C41))</f>
         <v/>
       </c>
       <c r="D41" s="20" t="str">
@@ -6956,15 +6950,15 @@
         <v>Oquelí Domínguez Murdered in Guapinol</v>
       </c>
       <c r="E41" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E41), "", CONCAT("http://localhost:4040/", Sources!E41))</f>
-        <v>http://localhost:4040/images/15062023.jpg</v>
+        <f>IF(ISBLANK(Sources!E41), "", CONCAT("", Sources!E41))</f>
+        <v>images/15062023.jpg</v>
       </c>
       <c r="F41" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F41), "", CONCAT("http://localhost:4040/", Sources!F41))</f>
+        <f>IF(ISBLANK(Sources!F41), "", CONCAT("", Sources!F41))</f>
         <v/>
       </c>
       <c r="G41" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G41), "", CONCAT("http://localhost:4040/", Sources!G41))</f>
+        <f>IF(ISBLANK(Sources!G41), "", CONCAT("", Sources!G41))</f>
         <v/>
       </c>
     </row>
@@ -6978,7 +6972,7 @@
         <v>Public Assembly on Los Pinares Project Prematurely Suspended</v>
       </c>
       <c r="C42" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C42), "", CONCAT("http://localhost:4040/images/", Sources!C42))</f>
+        <f>IF(ISBLANK(Sources!C42), "", CONCAT("images/", Sources!C42))</f>
         <v/>
       </c>
       <c r="D42" s="20" t="str">
@@ -6986,15 +6980,15 @@
         <v>Public Assembly on Los Pinares Project Prematurely Suspended</v>
       </c>
       <c r="E42" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E42), "", CONCAT("http://localhost:4040/", Sources!E42))</f>
-        <v>http://localhost:4040/images/09122023.jpg</v>
+        <f>IF(ISBLANK(Sources!E42), "", CONCAT("", Sources!E42))</f>
+        <v>images/09122023.jpg</v>
       </c>
       <c r="F42" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F42), "", CONCAT("http://localhost:4040/", Sources!F42))</f>
+        <f>IF(ISBLANK(Sources!F42), "", CONCAT("", Sources!F42))</f>
         <v/>
       </c>
       <c r="G42" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G42), "", CONCAT("http://localhost:4040/", Sources!G42))</f>
+        <f>IF(ISBLANK(Sources!G42), "", CONCAT("", Sources!G42))</f>
         <v/>
       </c>
     </row>
@@ -7008,7 +7002,7 @@
         <v>Mining Concession Permits Expire and Protests Organized</v>
       </c>
       <c r="C43" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C43), "", CONCAT("http://localhost:4040/images/", Sources!C43))</f>
+        <f>IF(ISBLANK(Sources!C43), "", CONCAT("images/", Sources!C43))</f>
         <v/>
       </c>
       <c r="D43" s="20" t="str">
@@ -7016,15 +7010,15 @@
         <v>Mining Concession Permits Expire and Protests Organized</v>
       </c>
       <c r="E43" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E43), "", CONCAT("http://localhost:4040/", Sources!E43))</f>
-        <v>http://localhost:4040/images/28012024.mp4</v>
-      </c>
-      <c r="F43" s="32" t="str">
-        <f>IF(ISBLANK(Sources!F43), "", CONCAT("http://localhost:4040/", Sources!F43))</f>
-        <v>http://localhost:4040/images/28012024a.jpg</v>
+        <f>IF(ISBLANK(Sources!E43), "", CONCAT("", Sources!E43))</f>
+        <v>images/28012024.mp4</v>
+      </c>
+      <c r="F43" s="20" t="str">
+        <f>IF(ISBLANK(Sources!F43), "", CONCAT("", Sources!F43))</f>
+        <v>images/28012024a.jpg</v>
       </c>
       <c r="G43" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G43), "", CONCAT("http://localhost:4040/", Sources!G43))</f>
+        <f>IF(ISBLANK(Sources!G43), "", CONCAT("", Sources!G43))</f>
         <v/>
       </c>
     </row>
@@ -7038,7 +7032,7 @@
         <v>Second Public Assembly Suspended Following Legal Appeal</v>
       </c>
       <c r="C44" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C44), "", CONCAT("http://localhost:4040/images/", Sources!C44))</f>
+        <f>IF(ISBLANK(Sources!C44), "", CONCAT("images/", Sources!C44))</f>
         <v/>
       </c>
       <c r="D44" s="20" t="str">
@@ -7046,15 +7040,15 @@
         <v>Second Public Assembly Suspended Following Legal Appeal</v>
       </c>
       <c r="E44" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E44), "", CONCAT("http://localhost:4040/", Sources!E44))</f>
-        <v>http://localhost:4040/images/31012024.jpg</v>
+        <f>IF(ISBLANK(Sources!E44), "", CONCAT("", Sources!E44))</f>
+        <v>images/31012024.jpg</v>
       </c>
       <c r="F44" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F44), "", CONCAT("http://localhost:4040/", Sources!F44))</f>
+        <f>IF(ISBLANK(Sources!F44), "", CONCAT("", Sources!F44))</f>
         <v/>
       </c>
       <c r="G44" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G44), "", CONCAT("http://localhost:4040/", Sources!G44))</f>
+        <f>IF(ISBLANK(Sources!G44), "", CONCAT("", Sources!G44))</f>
         <v/>
       </c>
     </row>
@@ -7068,7 +7062,7 @@
         <v>Petroleum Coke Plant Approved Amid Community Opposition</v>
       </c>
       <c r="C45" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C45), "", CONCAT("http://localhost:4040/images/", Sources!C45))</f>
+        <f>IF(ISBLANK(Sources!C45), "", CONCAT("images/", Sources!C45))</f>
         <v/>
       </c>
       <c r="D45" s="20" t="str">
@@ -7076,15 +7070,15 @@
         <v>Petroleum Coke Plant Approved Amid Community Opposition</v>
       </c>
       <c r="E45" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E45), "", CONCAT("http://localhost:4040/", Sources!E45))</f>
-        <v>http://localhost:4040/images/13062024.jpg</v>
-      </c>
-      <c r="F45" s="32" t="str">
-        <f>IF(ISBLANK(Sources!F45), "", CONCAT("http://localhost:4040/", Sources!F45))</f>
-        <v>http://localhost:4040/images/13062024a.mp4</v>
+        <f>IF(ISBLANK(Sources!E45), "", CONCAT("", Sources!E45))</f>
+        <v>images/13062024.jpg</v>
+      </c>
+      <c r="F45" s="20" t="str">
+        <f>IF(ISBLANK(Sources!F45), "", CONCAT("", Sources!F45))</f>
+        <v>images/13062024a.mp4</v>
       </c>
       <c r="G45" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G45), "", CONCAT("http://localhost:4040/", Sources!G45))</f>
+        <f>IF(ISBLANK(Sources!G45), "", CONCAT("", Sources!G45))</f>
         <v/>
       </c>
     </row>
@@ -7098,7 +7092,7 @@
         <v>Government Restores Original Carlos Escaleras National Park Boundaries</v>
       </c>
       <c r="C46" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C46), "", CONCAT("http://localhost:4040/images/", Sources!C46))</f>
+        <f>IF(ISBLANK(Sources!C46), "", CONCAT("images/", Sources!C46))</f>
         <v/>
       </c>
       <c r="D46" s="20" t="str">
@@ -7106,15 +7100,15 @@
         <v>Government Restores Original Carlos Escaleras National Park Boundaries</v>
       </c>
       <c r="E46" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E46), "", CONCAT("http://localhost:4040/", Sources!E46))</f>
+        <f>IF(ISBLANK(Sources!E46), "", CONCAT("", Sources!E46))</f>
         <v/>
       </c>
       <c r="F46" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F46), "", CONCAT("http://localhost:4040/", Sources!F46))</f>
+        <f>IF(ISBLANK(Sources!F46), "", CONCAT("", Sources!F46))</f>
         <v/>
       </c>
       <c r="G46" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G46), "", CONCAT("http://localhost:4040/", Sources!G46))</f>
+        <f>IF(ISBLANK(Sources!G46), "", CONCAT("", Sources!G46))</f>
         <v/>
       </c>
     </row>
@@ -7128,7 +7122,7 @@
         <v>CMDBCP Coordinator Juan López Assassinated</v>
       </c>
       <c r="C47" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C47), "", CONCAT("http://localhost:4040/images/", Sources!C47))</f>
+        <f>IF(ISBLANK(Sources!C47), "", CONCAT("images/", Sources!C47))</f>
         <v/>
       </c>
       <c r="D47" s="20" t="str">
@@ -7136,15 +7130,15 @@
         <v>CMDBCP Coordinator Juan López Assassinated</v>
       </c>
       <c r="E47" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E47), "", CONCAT("http://localhost:4040/", Sources!E47))</f>
-        <v>http://localhost:4040/images/14092024.jpg</v>
+        <f>IF(ISBLANK(Sources!E47), "", CONCAT("", Sources!E47))</f>
+        <v>images/14092024.jpg</v>
       </c>
       <c r="F47" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F47), "", CONCAT("http://localhost:4040/", Sources!F47))</f>
+        <f>IF(ISBLANK(Sources!F47), "", CONCAT("", Sources!F47))</f>
         <v/>
       </c>
       <c r="G47" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G47), "", CONCAT("http://localhost:4040/", Sources!G47))</f>
+        <f>IF(ISBLANK(Sources!G47), "", CONCAT("", Sources!G47))</f>
         <v/>
       </c>
     </row>
@@ -7158,7 +7152,7 @@
         <v>Criminal Proceedings Reopened Against CMDBCP Members</v>
       </c>
       <c r="C48" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C48), "", CONCAT("http://localhost:4040/images/", Sources!C48))</f>
+        <f>IF(ISBLANK(Sources!C48), "", CONCAT("images/", Sources!C48))</f>
         <v/>
       </c>
       <c r="D48" s="20" t="str">
@@ -7166,15 +7160,15 @@
         <v>Criminal Proceedings Reopened Against CMDBCP Members</v>
       </c>
       <c r="E48" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E48), "", CONCAT("http://localhost:4040/", Sources!E48))</f>
+        <f>IF(ISBLANK(Sources!E48), "", CONCAT("", Sources!E48))</f>
         <v/>
       </c>
       <c r="F48" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F48), "", CONCAT("http://localhost:4040/", Sources!F48))</f>
+        <f>IF(ISBLANK(Sources!F48), "", CONCAT("", Sources!F48))</f>
         <v/>
       </c>
       <c r="G48" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G48), "", CONCAT("http://localhost:4040/", Sources!G48))</f>
+        <f>IF(ISBLANK(Sources!G48), "", CONCAT("", Sources!G48))</f>
         <v/>
       </c>
     </row>
@@ -7188,7 +7182,7 @@
         <v>Definitive Freedom Granted to Remaining Defendants</v>
       </c>
       <c r="C49" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C49), "", CONCAT("http://localhost:4040/images/", Sources!C49))</f>
+        <f>IF(ISBLANK(Sources!C49), "", CONCAT("images/", Sources!C49))</f>
         <v/>
       </c>
       <c r="D49" s="20" t="str">
@@ -7196,15 +7190,15 @@
         <v>Definitive Freedom Granted to Remaining Defendants</v>
       </c>
       <c r="E49" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E49), "", CONCAT("http://localhost:4040/", Sources!E49))</f>
+        <f>IF(ISBLANK(Sources!E49), "", CONCAT("", Sources!E49))</f>
         <v/>
       </c>
       <c r="F49" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F49), "", CONCAT("http://localhost:4040/", Sources!F49))</f>
+        <f>IF(ISBLANK(Sources!F49), "", CONCAT("", Sources!F49))</f>
         <v/>
       </c>
       <c r="G49" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G49), "", CONCAT("http://localhost:4040/", Sources!G49))</f>
+        <f>IF(ISBLANK(Sources!G49), "", CONCAT("", Sources!G49))</f>
         <v/>
       </c>
     </row>
@@ -7218,7 +7212,7 @@
         <v>Mayor Adán Fúnez Identified as Person of Interest in Murder Case</v>
       </c>
       <c r="C50" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C50), "", CONCAT("http://localhost:4040/images/", Sources!C50))</f>
+        <f>IF(ISBLANK(Sources!C50), "", CONCAT("images/", Sources!C50))</f>
         <v/>
       </c>
       <c r="D50" s="20" t="str">
@@ -7226,15 +7220,15 @@
         <v>Mayor Adán Fúnez Identified as Person of Interest in Murder Case</v>
       </c>
       <c r="E50" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E50), "", CONCAT("http://localhost:4040/", Sources!E50))</f>
+        <f>IF(ISBLANK(Sources!E50), "", CONCAT("", Sources!E50))</f>
         <v/>
       </c>
       <c r="F50" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F50), "", CONCAT("http://localhost:4040/", Sources!F50))</f>
+        <f>IF(ISBLANK(Sources!F50), "", CONCAT("", Sources!F50))</f>
         <v/>
       </c>
       <c r="G50" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G50), "", CONCAT("http://localhost:4040/", Sources!G50))</f>
+        <f>IF(ISBLANK(Sources!G50), "", CONCAT("", Sources!G50))</f>
         <v/>
       </c>
     </row>
@@ -7248,7 +7242,7 @@
         <v>Residents Call for Los Pinares Expulsion and Justice for Juan López</v>
       </c>
       <c r="C51" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C51), "", CONCAT("http://localhost:4040/images/", Sources!C51))</f>
+        <f>IF(ISBLANK(Sources!C51), "", CONCAT("images/", Sources!C51))</f>
         <v/>
       </c>
       <c r="D51" s="20" t="str">
@@ -7256,15 +7250,15 @@
         <v>Residents Call for Los Pinares Expulsion and Justice for Juan López</v>
       </c>
       <c r="E51" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E51), "", CONCAT("http://localhost:4040/", Sources!E51))</f>
-        <v>http://localhost:4040/images/26022025.mp4</v>
+        <f>IF(ISBLANK(Sources!E51), "", CONCAT("", Sources!E51))</f>
+        <v>images/26022025.mp4</v>
       </c>
       <c r="F51" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F51), "", CONCAT("http://localhost:4040/", Sources!F51))</f>
+        <f>IF(ISBLANK(Sources!F51), "", CONCAT("", Sources!F51))</f>
         <v/>
       </c>
       <c r="G51" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G51), "", CONCAT("http://localhost:4040/", Sources!G51))</f>
+        <f>IF(ISBLANK(Sources!G51), "", CONCAT("", Sources!G51))</f>
         <v/>
       </c>
     </row>
@@ -7278,7 +7272,7 @@
         <v>Los Pinares Executives Summoned to Court on Criminal Charges</v>
       </c>
       <c r="C52" s="30" t="str">
-        <f>IF(ISBLANK(Sources!C52), "", CONCAT("http://localhost:4040/images/", Sources!C52))</f>
+        <f>IF(ISBLANK(Sources!C52), "", CONCAT("images/", Sources!C52))</f>
         <v/>
       </c>
       <c r="D52" s="20" t="str">
@@ -7286,15 +7280,15 @@
         <v>Los Pinares Executives Summoned to Court on Criminal Charges</v>
       </c>
       <c r="E52" s="31" t="str">
-        <f>IF(ISBLANK(Sources!E52), "", CONCAT("http://localhost:4040/", Sources!E52))</f>
-        <v>http://localhost:4040/images/28022025.jpg</v>
+        <f>IF(ISBLANK(Sources!E52), "", CONCAT("", Sources!E52))</f>
+        <v>images/28022025.jpg</v>
       </c>
       <c r="F52" s="20" t="str">
-        <f>IF(ISBLANK(Sources!F52), "", CONCAT("http://localhost:4040/", Sources!F52))</f>
+        <f>IF(ISBLANK(Sources!F52), "", CONCAT("", Sources!F52))</f>
         <v/>
       </c>
       <c r="G52" s="20" t="str">
-        <f>IF(ISBLANK(Sources!G52), "", CONCAT("http://localhost:4040/", Sources!G52))</f>
+        <f>IF(ISBLANK(Sources!G52), "", CONCAT("", Sources!G52))</f>
         <v/>
       </c>
     </row>
@@ -7321,7 +7315,7 @@
       <c r="A1" s="18" t="s">
         <v>272</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="32" t="s">
         <v>273</v>
       </c>
       <c r="C1" s="18" t="s">
@@ -7391,7 +7385,7 @@
         <f>Associations!D3</f>
         <v/>
       </c>
-      <c r="F3" s="34" t="str">
+      <c r="F3" s="33" t="str">
         <f>Associations!E3</f>
         <v/>
       </c>
@@ -7418,7 +7412,7 @@
         <f>Associations!D4</f>
         <v/>
       </c>
-      <c r="F4" s="34" t="str">
+      <c r="F4" s="33" t="str">
         <f>Associations!E4</f>
         <v/>
       </c>
@@ -7445,7 +7439,7 @@
         <f>Associations!D5</f>
         <v/>
       </c>
-      <c r="F5" s="34" t="str">
+      <c r="F5" s="33" t="str">
         <f>Associations!E5</f>
         <v/>
       </c>
@@ -7472,7 +7466,7 @@
         <f>Associations!D6</f>
         <v/>
       </c>
-      <c r="F6" s="34" t="str">
+      <c r="F6" s="33" t="str">
         <f>Associations!E6</f>
         <v/>
       </c>
@@ -7499,7 +7493,7 @@
         <f>Associations!D7</f>
         <v/>
       </c>
-      <c r="F7" s="34" t="str">
+      <c r="F7" s="33" t="str">
         <f>Associations!E7</f>
         <v/>
       </c>
@@ -7526,7 +7520,7 @@
         <f>Associations!D8</f>
         <v/>
       </c>
-      <c r="F8" s="34" t="str">
+      <c r="F8" s="33" t="str">
         <f>Associations!E8</f>
         <v/>
       </c>
@@ -7553,7 +7547,7 @@
         <f>Associations!D9</f>
         <v/>
       </c>
-      <c r="F9" s="34" t="str">
+      <c r="F9" s="33" t="str">
         <f>Associations!E9</f>
         <v/>
       </c>
@@ -7580,7 +7574,7 @@
         <f>Associations!D10</f>
         <v/>
       </c>
-      <c r="F10" s="34" t="str">
+      <c r="F10" s="33" t="str">
         <f>Associations!E10</f>
         <v/>
       </c>
@@ -7607,7 +7601,7 @@
         <f>Associations!D11</f>
         <v/>
       </c>
-      <c r="F11" s="34" t="str">
+      <c r="F11" s="33" t="str">
         <f>Associations!E11</f>
         <v/>
       </c>

</xml_diff>